<commit_message>
Auto update XML, XLSX archive and MD5
</commit_message>
<xml_diff>
--- a/datasets/klebark/archive/ceny_2026-09-30.xlsx
+++ b/datasets/klebark/archive/ceny_2026-09-30.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB101A74-73B6-4DAB-925D-4C57452D0291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C531E1-FFD2-4B97-8615-079C5B79A3FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23040" yWindow="120" windowWidth="29040" windowHeight="13680" xr2:uid="{336D2583-5C4C-4C42-9206-61D546232E49}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{336D2583-5C4C-4C42-9206-61D546232E49}"/>
   </bookViews>
   <sheets>
     <sheet name="wzorcowy zakres danych" sheetId="7" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="674" uniqueCount="85">
   <si>
     <t>Nazwa dewelopera</t>
   </si>
@@ -816,7 +816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA33353A-1A07-421F-B982-7CDBB172178E}">
-  <dimension ref="A1:BF19"/>
+  <dimension ref="A1:BF18"/>
   <sheetFormatPr defaultColWidth="27.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="6" width="27.7109375" style="1"/>
@@ -3402,7 +3402,7 @@
         <v>70</v>
       </c>
       <c r="AH15" s="21">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="AI15" s="4" t="s">
         <v>71</v>
@@ -3411,7 +3411,7 @@
         <v>74</v>
       </c>
       <c r="AK15" s="12" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="AL15" s="20">
         <v>6722</v>
@@ -3426,7 +3426,7 @@
         <v>46205</v>
       </c>
       <c r="AP15" s="19">
-        <v>920886.5</v>
+        <v>910432</v>
       </c>
       <c r="AQ15" s="14">
         <v>46205</v>
@@ -3477,198 +3477,22 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:58" s="7" customFormat="1" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C16" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="E16" s="3">
-        <v>1132874423</v>
-      </c>
-      <c r="F16" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="G16" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="I16" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O16" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="P16" s="3">
-        <v>5</v>
-      </c>
-      <c r="Q16" s="3">
-        <v>10</v>
-      </c>
-      <c r="R16" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="S16" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="T16" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="U16" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="V16" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="W16" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="X16" s="5">
-        <v>16</v>
-      </c>
-      <c r="Y16" s="3">
-        <v>2</v>
-      </c>
-      <c r="Z16" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="AA16" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB16" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="AC16" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD16" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE16" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="AF16" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG16" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AH16" s="21">
-        <v>13</v>
-      </c>
-      <c r="AI16" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AJ16" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK16" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="AL16" s="20">
-        <v>6722</v>
-      </c>
-      <c r="AM16" s="14">
-        <v>46205</v>
-      </c>
-      <c r="AN16" s="19">
-        <v>899000</v>
-      </c>
-      <c r="AO16" s="14">
-        <v>46205</v>
-      </c>
-      <c r="AP16" s="19">
-        <v>910432</v>
-      </c>
-      <c r="AQ16" s="14">
-        <v>46205</v>
-      </c>
-      <c r="AR16" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="AS16" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="AT16" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="AU16" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="AV16" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="AW16" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="AX16" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="AY16" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="AZ16" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="BA16" s="19">
-        <v>1000</v>
-      </c>
-      <c r="BB16" s="14">
-        <v>44424</v>
-      </c>
-      <c r="BC16" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="BD16" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="BE16" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="BF16" s="18" t="s">
-        <v>82</v>
-      </c>
+    <row r="16" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="AN16" s="30"/>
+      <c r="AO16" s="31"/>
+      <c r="AX16" s="30"/>
+      <c r="AZ16" s="32"/>
+      <c r="BD16" s="30"/>
+      <c r="BF16" s="33"/>
     </row>
     <row r="17" spans="40:58" x14ac:dyDescent="0.25">
       <c r="AN17" s="30"/>
       <c r="AO17" s="31"/>
-      <c r="AX17" s="30"/>
-      <c r="AZ17" s="32"/>
-      <c r="BD17" s="30"/>
       <c r="BF17" s="33"/>
     </row>
     <row r="18" spans="40:58" x14ac:dyDescent="0.25">
-      <c r="AN18" s="30"/>
       <c r="AO18" s="31"/>
       <c r="BF18" s="33"/>
-    </row>
-    <row r="19" spans="40:58" x14ac:dyDescent="0.25">
-      <c r="AO19" s="31"/>
-      <c r="BF19" s="33"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>